<commit_message>
allow double booking instructors in case of partners
</commit_message>
<xml_diff>
--- a/Data/Course Catalog_Master Tracker for 2027_062826_for Schedule Pro OW.xlsx
+++ b/Data/Course Catalog_Master Tracker for 2027_062826_for Schedule Pro OW.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/o/SchedulePro2/SchedulePro2/Data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{E786BED6-85F9-FA4D-8307-7FD7D4BF71E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{05C50FC2-1EA2-4B41-814E-458B4727FD2D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="15280" yWindow="-26700" windowWidth="23800" windowHeight="24980" tabRatio="707" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-11480" yWindow="-28200" windowWidth="25600" windowHeight="28200" tabRatio="707" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Course Info 2027" sheetId="12" r:id="rId1"/>
@@ -121,7 +121,7 @@
           <rPr>
             <b/>
             <sz val="9"/>
-            <color indexed="81"/>
+            <color rgb="FF000000"/>
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
@@ -130,12 +130,21 @@
         <r>
           <rPr>
             <sz val="9"/>
-            <color indexed="81"/>
+            <color rgb="FF000000"/>
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
           <t xml:space="preserve">
-Please note change from prior years to a 31 capacity.</t>
+</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Please note change from prior years to a 31 capacity.</t>
         </r>
       </text>
     </comment>
@@ -145,7 +154,7 @@
           <rPr>
             <b/>
             <sz val="9"/>
-            <color indexed="81"/>
+            <color rgb="FF000000"/>
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
@@ -154,12 +163,21 @@
         <r>
           <rPr>
             <sz val="9"/>
-            <color indexed="81"/>
+            <color rgb="FF000000"/>
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
           <t xml:space="preserve">
-Called "Project Management" on the CCR sheet</t>
+</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Called "Project Management" on the CCR sheet</t>
         </r>
       </text>
     </comment>
@@ -643,12 +661,21 @@
         <r>
           <rPr>
             <sz val="11"/>
-            <color theme="1"/>
+            <color rgb="FF000000"/>
             <rFont val="Calibri"/>
             <family val="2"/>
-            <scheme val="minor"/>
           </rPr>
           <t xml:space="preserve">Samantha Mulford:Verify that 8th edition update is occurring and ensure Content License in place.
+</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="11"/>
+            <color rgb="FF000000"/>
+            <rFont val="Calibri"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
 </t>
         </r>
       </text>
@@ -9951,7 +9978,7 @@
     <numFmt numFmtId="44" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="164" formatCode="00000"/>
   </numFmts>
-  <fonts count="25">
+  <fonts count="27">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -10116,6 +10143,19 @@
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="9"/>
+      <color rgb="FF000000"/>
+      <name val="Tahoma"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color rgb="FF000000"/>
+      <name val="Tahoma"/>
       <family val="2"/>
     </font>
   </fonts>
@@ -33300,6 +33340,33 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="317a123e-8a65-4dab-bc2c-6fce56555643">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="be60641a-447f-4dc1-b472-18eab195af2e" xsi:nil="true"/>
+    <SharedWithUsers xmlns="be60641a-447f-4dc1-b472-18eab195af2e">
+      <UserInfo>
+        <DisplayName/>
+        <AccountId xsi:nil="true"/>
+        <AccountType/>
+      </UserInfo>
+    </SharedWithUsers>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100B3AC32CE7CC0584E8A3F35A29B9B27E4" ma:contentTypeVersion="22" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="73f7271cafb0ecafdc6982455c2b93c0">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="317a123e-8a65-4dab-bc2c-6fce56555643" xmlns:ns3="be60641a-447f-4dc1-b472-18eab195af2e" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="7cd34201f59828bcf7f2e792e20dad91" ns2:_="" ns3:_="">
     <xsd:import namespace="317a123e-8a65-4dab-bc2c-6fce56555643"/>
@@ -33540,48 +33607,10 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="317a123e-8a65-4dab-bc2c-6fce56555643">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="be60641a-447f-4dc1-b472-18eab195af2e" xsi:nil="true"/>
-    <SharedWithUsers xmlns="be60641a-447f-4dc1-b472-18eab195af2e">
-      <UserInfo>
-        <DisplayName/>
-        <AccountId xsi:nil="true"/>
-        <AccountType/>
-      </UserInfo>
-    </SharedWithUsers>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E0D2758E-9245-495A-9DA4-1B0F3EF7900F}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C1FE27D4-AB8F-464A-B6FB-FB4BD2D08AFF}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="317a123e-8a65-4dab-bc2c-6fce56555643"/>
-    <ds:schemaRef ds:uri="be60641a-447f-4dc1-b472-18eab195af2e"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -33604,9 +33633,20 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C1FE27D4-AB8F-464A-B6FB-FB4BD2D08AFF}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E0D2758E-9245-495A-9DA4-1B0F3EF7900F}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="317a123e-8a65-4dab-bc2c-6fce56555643"/>
+    <ds:schemaRef ds:uri="be60641a-447f-4dc1-b472-18eab195af2e"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>